<commit_message>
feat(inventory): add consumable lot details and expiry notifications in VatTuDetailsSheet
feat(transactions): implement TransactionDetailSheet for detailed transaction view

feat(campaign): add campaign status metadata fetching and update campaign status types

feat(depot): add advance limit configuration for depots

fix(ui): adjust card padding for better layout

fix(inventory): handle optional reusable breakdown properties in VatTuTabContent

refactor(api): enhance inventory and campaign APIs for better data handling

chore(templates): update inventory templates for improved usability
</commit_message>
<xml_diff>
--- a/public/templates/mau_nhap_kho_thuong.xlsx
+++ b/public/templates/mau_nhap_kho_thuong.xlsx
@@ -9,6 +9,10 @@
   <sheets>
     <sheet name="Template" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="TaiSuDung">Template!$M$5</definedName>
+    <definedName name="TieuThu">Template!$L$5:$L$9</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -27,7 +31,13 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+  <si>
+    <t>MẪU NHẬP KHO THƯỜNG</t>
+  </si>
+  <si>
+    <t>* Lưu ý: Đối với vật phẩm ‘Tái sử dụng’, đối tượng áp dụng thuộc nhóm ‘Lực lượng cứu hộ’.</t>
+  </si>
   <si>
     <t>STT</t>
   </si>
@@ -47,9 +57,6 @@
     <t>Đơn vị</t>
   </si>
   <si>
-    <t>Đơn giá</t>
-  </si>
-  <si>
     <t>Số lượng</t>
   </si>
   <si>
@@ -66,16 +73,49 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="41" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="42" formatCode="_-&quot;£&quot;* #,##0_-;\-&quot;£&quot;* #,##0_-;_-&quot;£&quot;* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="44" formatCode="_-&quot;£&quot;* #,##0.00_-;\-&quot;£&quot;* #,##0.00_-;_-&quot;£&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="176" formatCode="dd/mm/yyyy;@"/>
   </numFmts>
-  <fonts count="21">
+  <fonts count="25">
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
       <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -232,7 +272,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="35">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -241,6 +281,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="3" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FFFFFFCC"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -426,12 +478,27 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -535,153 +602,174 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="5" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="6" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="176" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="176" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="176" fontId="4" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1065,8 +1153,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:K6"/>
-  <sheetFormatPr defaultColWidth="7.94117647058824" defaultRowHeight="17.6" outlineLevelRow="5"/>
+  <dimension ref="A1:M21"/>
+  <sheetFormatPr defaultColWidth="7.94117647058824" defaultRowHeight="17.6"/>
   <cols>
     <col min="1" max="1" width="6.83088235294118" customWidth="1"/>
     <col min="2" max="2" width="25.8308823529412" customWidth="1"/>
@@ -1074,76 +1162,327 @@
     <col min="4" max="4" width="16.8308823529412" customWidth="1"/>
     <col min="5" max="5" width="18.8308823529412" customWidth="1"/>
     <col min="6" max="6" width="10.8308823529412" customWidth="1"/>
-    <col min="7" max="8" width="12.8308823529412" customWidth="1"/>
-    <col min="9" max="10" width="14.8308823529412" customWidth="1"/>
-    <col min="11" max="11" width="35.8308823529412" customWidth="1"/>
+    <col min="7" max="7" width="12.8308823529412" style="1" customWidth="1"/>
+    <col min="8" max="8" width="14.8308823529412" style="1" customWidth="1"/>
+    <col min="9" max="9" width="14.8308823529412" customWidth="1"/>
+    <col min="10" max="10" width="35.8308823529412" customWidth="1"/>
+    <col min="12" max="14" width="16.6470588235294" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
-      <c r="A1" t="s">
+    <row r="1" spans="1:10">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="7"/>
+      <c r="H1" s="7"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+    </row>
+    <row r="2" spans="1:10">
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="7"/>
+      <c r="H2" s="7"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
+      <c r="I3" s="4"/>
+      <c r="J3" s="4"/>
+    </row>
+    <row r="4" spans="1:13">
+      <c r="A4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B4" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="C4" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="D4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="E4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="G4" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="H4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="I4" s="5" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="2" spans="1:1">
-      <c r="A2">
+      <c r="J4" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L4" s="11"/>
+      <c r="M4" s="11"/>
+    </row>
+    <row r="5" spans="1:13">
+      <c r="A5" s="6">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1">
-      <c r="A3">
+      <c r="B5" s="6"/>
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="10"/>
+      <c r="H5" s="10"/>
+      <c r="I5" s="6"/>
+      <c r="J5" s="6"/>
+      <c r="L5" s="11"/>
+      <c r="M5" s="11"/>
+    </row>
+    <row r="6" spans="1:12">
+      <c r="A6" s="6">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1">
-      <c r="A4">
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="10"/>
+      <c r="H6" s="10"/>
+      <c r="I6" s="6"/>
+      <c r="J6" s="6"/>
+      <c r="L6" s="11"/>
+    </row>
+    <row r="7" spans="1:12">
+      <c r="A7" s="6">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1">
-      <c r="A5">
+      <c r="B7" s="6"/>
+      <c r="C7" s="6"/>
+      <c r="D7" s="6"/>
+      <c r="E7" s="6"/>
+      <c r="F7" s="6"/>
+      <c r="G7" s="10"/>
+      <c r="H7" s="10"/>
+      <c r="I7" s="6"/>
+      <c r="J7" s="6"/>
+      <c r="L7" s="11"/>
+    </row>
+    <row r="8" spans="1:12">
+      <c r="A8" s="6">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6">
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
+      <c r="G8" s="10"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="6"/>
+      <c r="J8" s="6"/>
+      <c r="L8" s="11"/>
+    </row>
+    <row r="9" spans="1:12">
+      <c r="A9" s="6">
         <v>5</v>
       </c>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
+      <c r="G9" s="10"/>
+      <c r="H9" s="10"/>
+      <c r="I9" s="6"/>
+      <c r="J9" s="6"/>
+      <c r="L9" s="11"/>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
+      <c r="G10" s="10"/>
+      <c r="H10" s="10"/>
+      <c r="I10" s="6"/>
+      <c r="J10" s="6"/>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="10"/>
+      <c r="I11" s="6"/>
+      <c r="J11" s="6"/>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
+      <c r="G12" s="10"/>
+      <c r="H12" s="10"/>
+      <c r="I12" s="6"/>
+      <c r="J12" s="6"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
+      <c r="G13" s="10"/>
+      <c r="H13" s="10"/>
+      <c r="I13" s="6"/>
+      <c r="J13" s="6"/>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="10"/>
+      <c r="H14" s="10"/>
+      <c r="I14" s="6"/>
+      <c r="J14" s="6"/>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
+      <c r="G15" s="10"/>
+      <c r="H15" s="10"/>
+      <c r="I15" s="6"/>
+      <c r="J15" s="6"/>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="10"/>
+      <c r="I16" s="6"/>
+      <c r="J16" s="6"/>
+    </row>
+    <row r="17" spans="1:10">
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
+      <c r="G17" s="10"/>
+      <c r="H17" s="10"/>
+      <c r="I17" s="6"/>
+      <c r="J17" s="6"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
+      <c r="G18" s="10"/>
+      <c r="H18" s="10"/>
+      <c r="I18" s="6"/>
+      <c r="J18" s="6"/>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
+      <c r="G19" s="10"/>
+      <c r="H19" s="10"/>
+      <c r="I19" s="6"/>
+      <c r="J19" s="6"/>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
+      <c r="G20" s="10"/>
+      <c r="H20" s="10"/>
+      <c r="I20" s="6"/>
+      <c r="J20" s="6"/>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
+      <c r="G21" s="10"/>
+      <c r="H21" s="10"/>
+      <c r="I21" s="6"/>
+      <c r="J21" s="6"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A3:J3"/>
+    <mergeCell ref="A1:J2"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C2 C5:C9 C11:C1048576">
+      <formula1>"Thực phẩm, Nước uống, Y tế, Vệ sinh cá nhân, Quần áo,Nơi trú ẩn, Công cụ sửa chữa, Thiết bị cứu hộ,Sưởi ấm,Phương tiện,Khác"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D1:D2 D5:D9 D11:D1048576">
+      <formula1>"Trẻ em, Người già,Phụ nữ mang thai,Chung,Lực lượng cứu hộ"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E1:E2 E5:E9 E11:E1048576">
+      <formula1>"Tiêu thụ,Tái sử dụng"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A2:A6 A1:F1 H1:K1" numberStoredAsText="1"/>
+    <ignoredError sqref="C1:C2 H$1:H$1048576" listDataValidation="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>